<commit_message>
Cập nhật bộ tài liệu báo cáo và nâng phiên bản Product Backlog
Rà soát, đồng bộ nội dung báo cáo tổng quan, proposal, user story, sprint backlog, test plan, test case, test report, reflection và báo cáo PDF tổng hợp.

Bổ sung bảng tính Test Report; cập nhật các bảng tính kiểm thử sprint 1, sprint 2 và sprint backlog.

Nâng Product Backlog từ phiên bản v1.3 lên v1.4, thay thế tệp phiên bản cũ.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BaoCao_Final/10.TestReport.xlsx
+++ b/BaoCao_Final/10.TestReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BaoCao_Final (2)\BaoCao_Final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="e:\Downloads\Document\BaoCao_Final(1)\BaoCao_Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50C2C0F2-782B-4E20-8BED-C2049549F5AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE2E6E4-AF0F-4D13-BD60-DFD96F96BAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestReportSprint1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="76">
   <si>
     <t>Test Report Sprint 2</t>
   </si>
@@ -696,21 +696,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:H33"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.81640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="34.81640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="58.36328125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.26953125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="20.1796875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="4.77734375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="34.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="58.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="20.21875" style="3" customWidth="1"/>
     <col min="6" max="6" width="14" style="3" customWidth="1"/>
     <col min="7" max="7" width="16" style="3" customWidth="1"/>
-    <col min="8" max="8" width="16.81640625" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" style="3"/>
+    <col min="8" max="8" width="16.77734375" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.77734375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="26.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:8" ht="26.55" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:8" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
         <v>28</v>
       </c>
@@ -721,7 +721,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
@@ -730,7 +730,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
@@ -738,10 +738,10 @@
         <v>4</v>
       </c>
       <c r="D5" s="11">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="10" t="s">
         <v>5</v>
@@ -750,16 +750,16 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
@@ -770,7 +770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
         <v>9</v>
@@ -779,7 +779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
         <v>10</v>
@@ -788,7 +788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
       <c r="C11" s="4" t="s">
         <v>11</v>
@@ -797,16 +797,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="15"/>
       <c r="D12" s="6">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" ht="33" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="33.6" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
         <v>13</v>
       </c>
@@ -829,7 +829,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
@@ -850,7 +850,7 @@
       </c>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
@@ -871,7 +871,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
@@ -892,7 +892,7 @@
       </c>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
@@ -913,7 +913,7 @@
       </c>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
@@ -934,7 +934,7 @@
       </c>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
@@ -955,7 +955,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
@@ -976,7 +976,7 @@
       </c>
       <c r="H21" s="1"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
@@ -997,7 +997,7 @@
       </c>
       <c r="H22" s="1"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="H23" s="1"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
         <v>49</v>
       </c>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="H25" s="1"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
         <v>51</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="7">
-        <v>0.9</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="F26" s="5">
         <v>0</v>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="H26" s="1"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B28" s="2" t="s">
         <v>21</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
         <v>67</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
         <v>70</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>71</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>20</v>
@@ -1132,31 +1132,31 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B31" s="14" t="s">
         <v>24</v>
       </c>
       <c r="C31" s="16"/>
-      <c r="D31" s="6" t="s">
-        <v>25</v>
+      <c r="D31" s="6">
+        <v>2</v>
       </c>
       <c r="E31" s="5">
         <v>1</v>
       </c>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
-      <c r="D32" s="6" t="s">
-        <v>26</v>
+      <c r="D32" s="6">
+        <v>0</v>
       </c>
       <c r="E32" s="5">
         <v>1</v>
       </c>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="6" t="s">
@@ -1173,28 +1173,29 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B31:C33"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="1.1811023622047243" right="0.59055118110236215" top="0.78740157480314954" bottom="0.78740157480314954" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9420FEE-2242-4A34-82C0-57D871DF8D4A}">
   <dimension ref="B1:H29"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.81640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="34.81640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="58.36328125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="20.1796875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="4.77734375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="34.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="58.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="20.21875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" style="3" customWidth="1"/>
     <col min="7" max="7" width="16" style="3" customWidth="1"/>
-    <col min="8" max="8" width="16.81640625" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" style="3"/>
+    <col min="8" max="8" width="16.77734375" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.77734375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="26.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:8" ht="26.55" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:8" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
         <v>0</v>
       </c>
@@ -1205,7 +1206,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
@@ -1214,7 +1215,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
@@ -1222,10 +1223,10 @@
         <v>4</v>
       </c>
       <c r="D5" s="11">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="10" t="s">
         <v>5</v>
@@ -1234,16 +1235,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="6">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1254,7 +1255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
         <v>9</v>
@@ -1263,7 +1264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
         <v>10</v>
@@ -1272,7 +1273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
       <c r="C11" s="4" t="s">
         <v>11</v>
@@ -1281,16 +1282,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="15"/>
       <c r="D12" s="6">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" ht="33" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="33.6" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
         <v>13</v>
       </c>
@@ -1313,7 +1314,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>53</v>
       </c>
@@ -1334,7 +1335,7 @@
       </c>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>55</v>
       </c>
@@ -1355,7 +1356,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>57</v>
       </c>
@@ -1376,7 +1377,7 @@
       </c>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>59</v>
       </c>
@@ -1397,7 +1398,7 @@
       </c>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>61</v>
       </c>
@@ -1418,7 +1419,7 @@
       </c>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>63</v>
       </c>
@@ -1439,7 +1440,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>65</v>
       </c>
@@ -1460,7 +1461,7 @@
       </c>
       <c r="H21" s="1"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
         <v>21</v>
       </c>
@@ -1477,7 +1478,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
         <v>55</v>
       </c>
@@ -1485,7 +1486,7 @@
         <v>72</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>73</v>
@@ -1494,7 +1495,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
         <v>57</v>
       </c>
@@ -1502,7 +1503,7 @@
         <v>74</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>73</v>
@@ -1511,7 +1512,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
         <v>61</v>
       </c>
@@ -1528,31 +1529,31 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B27" s="14" t="s">
         <v>24</v>
       </c>
       <c r="C27" s="16"/>
-      <c r="D27" s="6" t="s">
-        <v>25</v>
+      <c r="D27" s="6">
+        <v>0</v>
       </c>
       <c r="E27" s="5">
         <v>2</v>
       </c>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
-      <c r="D28" s="6" t="s">
-        <v>26</v>
+      <c r="D28" s="6">
+        <v>3</v>
       </c>
       <c r="E28" s="5">
         <v>1</v>
       </c>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="6" t="s">
@@ -1569,6 +1570,7 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B27:C29"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="1.1811023622047243" right="0.59055118110236215" top="0.78740157480314954" bottom="0.78740157480314954" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cập nhật đồng bộ bộ tài liệu báo cáo cuối kỳ
Cập nhật nội dung các tài liệu đề xuất, kế hoạch, user story, product backlog, thiết kế giao diện và quản lý cấu hình.

Làm mới bộ test plan, test case, test report, sprint backlog và biên bản họp; cập nhật báo cáo PDF.

Chuẩn hóa tên một số tài liệu Architecture, Sprint Backlog và Reflection; bổ sung tài liệu mở đầu, bản sao dự phòng, sơ đồ Database.drawio và gói BaoCao_Final.rar.

Xóa các phiên bản tài liệu cũ đã được thay thế.
</commit_message>
<xml_diff>
--- a/BaoCao_Final/10.TestReport.xlsx
+++ b/BaoCao_Final/10.TestReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="e:\Downloads\Document\BaoCao_Final(1)\BaoCao_Final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BaoCao_Final (5) - File Sửa\BaoCao_Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE2E6E4-AF0F-4D13-BD60-DFD96F96BAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC66200-CF08-4E74-96A0-3FED20A18AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestReportSprint1" sheetId="1" r:id="rId1"/>
@@ -696,21 +696,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:H33"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.77734375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="34.77734375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="58.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.21875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="20.21875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="4.81640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="34.81640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="58.36328125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="3" customWidth="1"/>
     <col min="6" max="6" width="14" style="3" customWidth="1"/>
     <col min="7" max="7" width="16" style="3" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.77734375" style="3"/>
+    <col min="8" max="8" width="16.81640625" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.81640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="26.55" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:8" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:8" ht="26.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="13" t="s">
         <v>28</v>
       </c>
@@ -721,7 +721,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
@@ -730,7 +730,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
@@ -741,7 +741,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" s="1"/>
       <c r="C6" s="10" t="s">
         <v>5</v>
@@ -750,7 +750,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="1"/>
       <c r="C7" s="4" t="s">
         <v>6</v>
@@ -759,7 +759,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
@@ -770,7 +770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
         <v>9</v>
@@ -779,7 +779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
         <v>10</v>
@@ -788,7 +788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="1"/>
       <c r="C11" s="4" t="s">
         <v>11</v>
@@ -797,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" s="14" t="s">
         <v>12</v>
       </c>
@@ -806,7 +806,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="33" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
         <v>13</v>
       </c>
@@ -829,7 +829,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
@@ -850,7 +850,7 @@
       </c>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
@@ -871,7 +871,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
@@ -892,7 +892,7 @@
       </c>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
@@ -913,7 +913,7 @@
       </c>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
@@ -934,7 +934,7 @@
       </c>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
@@ -955,7 +955,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
@@ -976,7 +976,7 @@
       </c>
       <c r="H21" s="1"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
@@ -997,7 +997,7 @@
       </c>
       <c r="H22" s="1"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="H23" s="1"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B25" s="1" t="s">
         <v>49</v>
       </c>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="H25" s="1"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B26" s="1" t="s">
         <v>51</v>
       </c>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="H26" s="1"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B28" s="2" t="s">
         <v>21</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
       <c r="B29" s="1" t="s">
         <v>67</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
       <c r="B30" s="1" t="s">
         <v>70</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B31" s="14" t="s">
         <v>24</v>
       </c>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
       <c r="D32" s="6">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="6" t="s">
@@ -1181,21 +1181,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9420FEE-2242-4A34-82C0-57D871DF8D4A}">
   <dimension ref="B1:H29"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.77734375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="34.77734375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="58.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="20.21875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="4.81640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="34.81640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="58.36328125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="19.90625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="20.1796875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13" style="3" customWidth="1"/>
     <col min="7" max="7" width="16" style="3" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.77734375" style="3"/>
+    <col min="8" max="8" width="16.81640625" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.81640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="26.55" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:8" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:8" ht="26.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="13" t="s">
         <v>0</v>
       </c>
@@ -1206,7 +1206,7 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
@@ -1226,7 +1226,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" s="1"/>
       <c r="C6" s="10" t="s">
         <v>5</v>
@@ -1235,7 +1235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="1"/>
       <c r="C7" s="4" t="s">
         <v>6</v>
@@ -1244,7 +1244,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1255,7 +1255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
         <v>9</v>
@@ -1264,7 +1264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
         <v>10</v>
@@ -1273,7 +1273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="1"/>
       <c r="C11" s="4" t="s">
         <v>11</v>
@@ -1282,7 +1282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" s="14" t="s">
         <v>12</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="33" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
         <v>13</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
         <v>53</v>
       </c>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="1" t="s">
         <v>55</v>
       </c>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B17" s="1" t="s">
         <v>57</v>
       </c>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B18" s="1" t="s">
         <v>59</v>
       </c>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B19" s="1" t="s">
         <v>61</v>
       </c>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B20" s="1" t="s">
         <v>63</v>
       </c>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B21" s="1" t="s">
         <v>65</v>
       </c>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="H21" s="1"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B23" s="2" t="s">
         <v>21</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
       <c r="B24" s="1" t="s">
         <v>55</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
       <c r="B25" s="1" t="s">
         <v>57</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="2:8" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" ht="49.5" x14ac:dyDescent="0.35">
       <c r="B26" s="1" t="s">
         <v>61</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B27" s="14" t="s">
         <v>24</v>
       </c>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
       <c r="D28" s="6">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="6" t="s">

</xml_diff>